<commit_message>
Show all committee affiliations in PVs; add affiliation columns to Excel template
Reported by Joel: Institution of Supervisor 2 and Examiner 1/2/3
affiliations were missing from generated PVs.

- New Student.supervisor_2_institution field (migration 0011)
- Import: explicit headers (Institution of Supervisor 2, President Jury
  Affiliation, Examiner N Affiliation) with fallbacks for legacy Coop
  files (duplicated 'Affiliation' columns); examiner 2/3 affiliations
  were previously never imported at all
- Template + sample xlsx now include every affiliation column
- PV Word & PDF: committee names rendered via a single shared helper
  covering co-supervisor and examiner 3; Supervisor/Co-Supervisor header
  lines now include the institution ('Name, UCAD, Senegal' format)
</commit_message>
<xml_diff>
--- a/defense/sample_data/test_with_idstudent.xlsx
+++ b/defense/sample_data/test_with_idstudent.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V32"/>
+  <dimension ref="A1:Z32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Affiliation </t>
+          <t>President Jury Affiliation</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Affiliation</t>
+          <t>Examiner 1 Affiliation</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
@@ -508,7 +508,7 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>Affiliation.1</t>
+          <t>Examiner 2 Affiliation</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
@@ -529,6 +529,26 @@
       <c r="V1" t="inlineStr">
         <is>
           <t>Email of Supervisor 2</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Institution of Supervisor 2</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Examiner 3</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Examiner 3 email</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Examiner 3 Affiliation</t>
         </is>
       </c>
     </row>
@@ -631,6 +651,10 @@
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -730,6 +754,10 @@
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -829,6 +857,10 @@
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -928,6 +960,10 @@
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1028,6 +1064,10 @@
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1126,6 +1166,10 @@
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1225,6 +1269,10 @@
       </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1323,6 +1371,10 @@
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1422,6 +1474,10 @@
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1522,6 +1578,10 @@
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1622,6 +1682,10 @@
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1721,6 +1785,10 @@
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1828,6 +1896,10 @@
           <t xml:space="preserve"> seydounourou.sylla@uadb.edu.sn</t>
         </is>
       </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1927,6 +1999,10 @@
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2027,6 +2103,10 @@
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2127,6 +2207,10 @@
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2227,6 +2311,10 @@
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2314,6 +2402,10 @@
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2413,6 +2505,10 @@
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2513,6 +2609,10 @@
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2612,6 +2712,10 @@
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2712,6 +2816,10 @@
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2819,6 +2927,10 @@
           <t xml:space="preserve"> seydounourou.sylla@uadb.edu.sn</t>
         </is>
       </c>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2920,6 +3032,10 @@
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3019,6 +3135,10 @@
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3121,6 +3241,10 @@
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3221,6 +3345,10 @@
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3319,6 +3447,10 @@
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3419,6 +3551,10 @@
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3519,6 +3655,10 @@
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3618,6 +3758,10 @@
       </c>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>